<commit_message>
chore: prepare dependencies and config for Streamlit Cloud deployment
</commit_message>
<xml_diff>
--- a/data/outreach_tracker.xlsx
+++ b/data/outreach_tracker.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,20 +478,124 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Mohit Decodes</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>mohitdecodes@gmail.com</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Collaboration on Fastapi with DevPulse</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Hi Mohit,
+Loved your recent breakdown on "FastAPI Full Course 2026 in Hindi | Beginner to Advanced | Projects + Interview Preparation". Your hands-on focus on Fastapi resonates deeply with our engineering team at DevPulse.
+We're launching an observability workspace built specifically for active developers. Given your engaged community, we would love to sponsor an upcoming video or partner on a dedicated community ambassador program.
+We provide full creative freedom and competitive rates. Would you be open to exploring a sponsorship or integration this month?
+Best regards,
+Alex Vance | DevPulse Partnerships</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Hey Mohit! Loved your recent breakdown on Fastapi. We're launching DevPulse and would love to partner on a collaboration. Open to a quick chat?</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-02 19:35:38</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FastAPI Master</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>support@fastapimaster.dev</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Collaboration on FastAPI with DevPulse</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Hi FastAPI,
+Loved your recent breakdown on "Building High Performance Asynchronous Background Tasks with FastAPI and Celery". Your hands-on focus on FastAPI resonates deeply with our engineering team at DevPulse.
+We're launching an observability workspace built specifically for active developers. Given your engaged community, we would love to sponsor an upcoming video or partner on a dedicated community ambassador program.
+We provide full creative freedom and competitive rates. Would you be open to exploring a sponsorship or integration this month?
+Best regards,
+Alex Vance | DevPulse Partnerships</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Hey FastAPI! Loved your recent breakdown on FastAPI. We're launching DevPulse and would love to partner on a collaboration. Open to a quick chat?</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Simulated</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-02 19:35:01</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SIMULATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>PromptLab with Leo</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>leo@promptlab.ai</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Collaboration on AI Agents with DevPulse</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Hi PromptLab,
 Loved your recent breakdown on "Building a Self-Correcting Research Agent with LangGraph and Python". Your hands-on focus on AI Agents resonates deeply with our engineering team at DevPulse.
@@ -501,49 +605,49 @@
 Alex Vance | DevPulse Partnerships</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Hey PromptLab! Loved your recent breakdown on AI Agents. We're launching DevPulse and would love to partner on a review. Open to a quick chat?</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026-10-02 03:38:59</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>SENT</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>AI Engineer Diary (Marta)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>marta@aiengineerdiary.dev</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Collaboration on LLMOps with DevPulse</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Hi AI,
 Loved your recent breakdown on "How We Test and Benchmark LLM Outputs Before Shipping to Production". Your hands-on focus on LLMOps resonates deeply with our engineering team at DevPulse.
@@ -553,27 +657,27 @@
 Alex Vance | DevPulse Partnerships</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Hey AI! Loved your recent breakdown on LLMOps. We're launching DevPulse and would love to partner on a collaboration. Open to a quick chat?</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Simulated</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>2026-10-02 02:29:02</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>SIMULATED</t>
         </is>

</xml_diff>